<commit_message>
sheoga trim: texture priced from the sheet; untexturable pieces ship smooth
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013k4uNVACPkQvSzK5uL9G1W
</commit_message>
<xml_diff>
--- a/src/testdata/sheoga-accessory-20261001.xlsx
+++ b/src/testdata/sheoga-accessory-20261001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\dataserver\Users\Logan\Desktop\Price Lists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F38DD9B-DC1D-425B-A77D-2EFDC7E86108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E8E883-9690-4B6C-839F-740F9E5B4B45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15943" xr2:uid="{6A2C4CCE-0550-47EA-A749-1D1CD558C496}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
   <si>
     <t>Shoe Mold</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>comes in 50LF bundles</t>
+  </si>
+  <si>
+    <t>Texture Charge</t>
+  </si>
+  <si>
+    <t>Cannot Be Textured</t>
   </si>
 </sst>
 </file>
@@ -191,7 +197,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -241,46 +247,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -343,69 +309,62 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -796,7 +755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{474E439D-B64E-472F-A7EA-8E96844A4C1B}">
-  <dimension ref="A3:Q32"/>
+  <dimension ref="A3:Q33"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="16.84375" bestFit="1" customWidth="1"/>
@@ -809,433 +768,459 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="13" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A4" s="5">
+      <c r="A4" s="3">
         <v>46296</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="20.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="25"/>
+      <c r="N13" s="25"/>
+      <c r="O13" s="25"/>
+      <c r="P13" s="25"/>
+      <c r="Q13" s="25"/>
     </row>
     <row r="15" spans="1:17" ht="18.45" x14ac:dyDescent="0.5">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="E15" s="11" t="s">
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="E15" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="11"/>
-      <c r="H15" s="11" t="s">
+      <c r="F15" s="21"/>
+      <c r="H15" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="I15" s="11"/>
-      <c r="K15" s="11" t="s">
+      <c r="I15" s="21"/>
+      <c r="K15" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="L15" s="11"/>
-      <c r="N15" s="6" t="s">
+      <c r="L15" s="21"/>
+      <c r="N15" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="O15" s="7"/>
+      <c r="O15" s="23"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="H16" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I16" s="12" t="s">
+      <c r="I16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="12" t="s">
+      <c r="K16" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L16" s="12" t="s">
+      <c r="L16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N16" s="8" t="s">
+      <c r="N16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="O16" s="9" t="s">
+      <c r="O16" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="6">
         <v>3.96</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="6">
         <v>5.98</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="6">
         <v>0.83</v>
       </c>
-      <c r="H17" s="12" t="s">
+      <c r="H17" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I17" s="14">
+      <c r="I17" s="6">
         <v>1.84</v>
       </c>
-      <c r="K17" s="12" t="s">
+      <c r="K17" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="L17" s="14">
+      <c r="L17" s="6">
         <v>1.28</v>
       </c>
-      <c r="N17" s="8" t="s">
+      <c r="N17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="O17" s="20">
+      <c r="O17" s="6">
         <v>0.1</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="14">
+      <c r="B18" s="6">
         <v>3.97</v>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="6">
         <v>6.43</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="6">
         <v>0.98</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="H18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I18" s="14">
+      <c r="I18" s="6">
         <v>2.21</v>
       </c>
-      <c r="K18" s="12" t="s">
+      <c r="K18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L18" s="14">
+      <c r="L18" s="6">
         <v>1.63</v>
       </c>
-      <c r="N18" s="8" t="s">
+      <c r="N18" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="O18" s="20">
+      <c r="O18" s="6">
         <v>0.15</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="14">
+      <c r="B19" s="6">
         <v>4.3</v>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="6">
         <v>6.89</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="14">
+      <c r="F19" s="6">
         <v>1.07</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="H19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="14">
+      <c r="I19" s="6">
         <v>2.39</v>
       </c>
-      <c r="K19" s="12" t="s">
+      <c r="K19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="L19" s="14">
+      <c r="L19" s="6">
         <v>1.67</v>
       </c>
-      <c r="N19" s="8" t="s">
+      <c r="N19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="O19" s="20">
+      <c r="O19" s="6">
         <v>0.2</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="6">
         <v>4.51</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="6">
         <v>6.79</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="6">
         <v>0.95</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="H20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I20" s="14">
+      <c r="I20" s="6">
         <v>2.09</v>
       </c>
-      <c r="K20" s="12" t="s">
+      <c r="K20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L20" s="14">
+      <c r="L20" s="6">
         <v>1.45</v>
       </c>
-      <c r="N20" s="10" t="s">
+      <c r="N20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="O20" s="21">
+      <c r="O20" s="6">
         <v>0.25</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="14">
+      <c r="B21" s="6">
         <v>3.61</v>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="6">
         <v>5.43</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="14">
+      <c r="F21" s="6">
         <v>0.75</v>
       </c>
-      <c r="H21" s="12" t="s">
+      <c r="H21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="14">
+      <c r="I21" s="6">
         <v>1.67</v>
       </c>
-      <c r="K21" s="12" t="s">
+      <c r="K21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="L21" s="14">
+      <c r="L21" s="6">
         <v>1.1599999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="6">
         <v>5.86</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="6">
         <v>9.4700000000000006</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F22" s="14">
+      <c r="F22" s="6">
         <v>1.36</v>
       </c>
-      <c r="H22" s="12" t="s">
+      <c r="H22" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I22" s="14">
+      <c r="I22" s="6">
         <v>3.03</v>
       </c>
-      <c r="K22" s="12" t="s">
+      <c r="K22" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="L22" s="14">
+      <c r="L22" s="6">
         <v>2.16</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="6">
         <v>7.04</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="6">
         <v>11.36</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F23" s="14">
+      <c r="F23" s="6">
         <v>1.63</v>
       </c>
-      <c r="H23" s="12" t="s">
+      <c r="H23" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I23" s="14">
+      <c r="I23" s="6">
         <v>3.63</v>
       </c>
-      <c r="K23" s="12" t="s">
+      <c r="K23" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L23" s="14">
+      <c r="L23" s="6">
         <v>2.59</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="23">
+      <c r="B24" s="9">
         <v>7.62</v>
       </c>
-      <c r="C24" s="23">
+      <c r="C24" s="9">
         <v>12.31</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="29">
+      <c r="F24" s="12">
         <v>1.76</v>
       </c>
-      <c r="H24" s="12" t="s">
+      <c r="H24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I24" s="14">
+      <c r="I24" s="6">
         <v>3.94</v>
       </c>
-      <c r="K24" s="12" t="s">
+      <c r="K24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L24" s="14">
+      <c r="L24" s="6">
         <v>2.81</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A25" s="26"/>
-      <c r="B25" s="27"/>
-      <c r="C25" s="28"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="15"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="15"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="15"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="20"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="7"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="7"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="7"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A26" s="24" t="s">
+      <c r="A26" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="25">
+      <c r="B26" s="11">
         <v>2.4</v>
       </c>
-      <c r="C26" s="25">
+      <c r="C26" s="11">
         <v>3.75</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="E26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F26" s="14">
+      <c r="F26" s="6">
         <v>1.85</v>
       </c>
-      <c r="H26" s="12" t="s">
+      <c r="H26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I26" s="14">
+      <c r="I26" s="6">
         <v>1.85</v>
       </c>
-      <c r="K26" s="12" t="s">
+      <c r="K26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L26" s="14">
+      <c r="L26" s="6">
         <v>1.85</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="6">
+        <v>2</v>
+      </c>
+      <c r="C27" s="6">
+        <v>2</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F27" s="15"/>
+      <c r="H27" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="I27" s="15"/>
+      <c r="K27" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="L27" s="15"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A28" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="18"/>
-      <c r="H27" s="17" t="s">
+      <c r="B28" s="16"/>
+      <c r="C28" s="15"/>
+      <c r="H28" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="I27" s="18"/>
-      <c r="K27" s="16" t="s">
+      <c r="I28" s="15"/>
+      <c r="K28" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="L27" s="16"/>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A29" s="2" t="s">
+      <c r="L28" s="17"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A30" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B30" s="2">
         <v>0.4</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A32" s="2" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A33" s="1" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="13">
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="A13:Q13"/>
+    <mergeCell ref="E27:F27"/>
     <mergeCell ref="H27:I27"/>
-    <mergeCell ref="A27:C27"/>
     <mergeCell ref="K27:L27"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="K28:L28"/>
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="K15:L15"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="A13:Q13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>